<commit_message>
Frontend update with verification and edit before download
</commit_message>
<xml_diff>
--- a/outputs/Residencial_Dom_Felipe_000000_seens.xlsx
+++ b/outputs/Residencial_Dom_Felipe_000000_seens.xlsx
@@ -474,7 +474,7 @@
     <row r="11">
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>(+) RECEITAS</t>
+          <t>(+) (+) RECEITAS</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
     <row r="14">
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>GS 2.560,67 6,85</t>
+          <t>GÁS 2.560,67 6,85</t>
         </is>
       </c>
       <c r="L14" s="3" t="n">
@@ -521,7 +521,7 @@
     <row r="16">
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>GUA 7.111,83 19,03</t>
+          <t>ÁGUA 7.111,83 19,03</t>
         </is>
       </c>
       <c r="L16" s="3" t="n">
@@ -591,7 +591,7 @@
     <row r="23">
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>(-) CONSERVA��O E MANUTEN��O</t>
+          <t>(-) CONSERVAÇÃO E MANUTENÇÃO</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
     <row r="27">
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t>(-) LIXO/DESINFETANTE/ �GUA SANIT�RIA /HIPOCLORITO</t>
+          <t>(-) MATERIAL DE LIMPEZA</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
     <row r="31">
       <c r="C31" s="1" t="inlineStr">
         <is>
-          <t>(-) TERRA</t>
+          <t>(-) (-) (-) (-) JARDINAGEM</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
     <row r="38">
       <c r="C38" s="1" t="inlineStr">
         <is>
-          <t>(-) DESPESAS ADMINISTRATIVAS</t>
+          <t>(-) (-) DESPESAS ADMINISTRATIVAS</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
     <row r="48">
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>GUA - SANEPAR - BLOCO A (27980473) CONS 159 M 01/2026 09/02/2026 DBITO AUT. 1.833,31</t>
+          <t>ÁGUA - SANEPAR - BLOCO A (27980473) CONS 159 M 01/2026 09/02/2026 DBITO AUT. 1.833,31</t>
         </is>
       </c>
       <c r="L48" s="3" t="n">
@@ -836,7 +836,7 @@
     <row r="49">
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>GUA - SANEPAR - BLOCO B (27980449) CONS 149 M 01/2026 09/02/2026 DBITO AUT. 1.802,60</t>
+          <t>ÁGUA - SANEPAR - BLOCO B (27980449) CONS 149 M 01/2026 09/02/2026 DBITO AUT. 1.802,60</t>
         </is>
       </c>
       <c r="L49" s="3" t="n">
@@ -846,7 +846,7 @@
     <row r="50">
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>GUA - SANEPAR - BLOCO C (27732488) CONS 126 M 01/2026 06/02/2026 DBITO AUT. 1.731,97</t>
+          <t>ÁGUA - SANEPAR - BLOCO C (27732488) CONS 126 M 01/2026 06/02/2026 DBITO AUT. 1.731,97</t>
         </is>
       </c>
       <c r="L50" s="3" t="n">
@@ -856,7 +856,7 @@
     <row r="51">
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>GUA - SANEPAR - BLOCO D (27732500) CONS 148 M 01/2026 06/02/2026 DBITO AUT. 1.743,89</t>
+          <t>ÁGUA - SANEPAR - BLOCO D (27732500) CONS 148 M 01/2026 06/02/2026 DBITO AUT. 1.743,89</t>
         </is>
       </c>
       <c r="L51" s="3" t="n">
@@ -866,7 +866,7 @@
     <row r="52">
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>GUA - SANEPAR - SALO (02616530) CONS 5 M 01/2026 09/02/2026 DBITO AUT. 99,42</t>
+          <t>ÁGUA - SANEPAR - SALO (02616530) CONS 5 M 01/2026 09/02/2026 DBITO AUT. 99,42</t>
         </is>
       </c>
       <c r="L52" s="3" t="n">
@@ -886,14 +886,14 @@
     <row r="54">
       <c r="C54" s="1" t="inlineStr">
         <is>
-          <t>(-) DESPESAS N�O RATEADAS</t>
+          <t>(-) (-) DESPESAS NÃO RATEADAS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>- AQUISIO DE UMA 11/2025 10/02/2026 BOLETO 10009 281,93</t>
+          <t>- AQUISIO DE UMA ROÇADEIRA 11/2025 10/02/2026 BOLETO 10009 281,93</t>
         </is>
       </c>
       <c r="L55" s="3" t="n">
@@ -913,7 +913,7 @@
     <row r="57">
       <c r="C57" s="1" t="inlineStr">
         <is>
-          <t>(-) RO�ADEIRA</t>
+          <t>(-) OUTROS MATERIAIS</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
     <row r="64">
       <c r="C64" s="1" t="inlineStr">
         <is>
-          <t>(-) M�VEIS E UTENS�LIOS</t>
+          <t>(-) MÓVEIS E UTENSÍLIOS</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1034,7 @@
     <row r="70">
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t>(-) DESPESAS BANC�RIAS</t>
+          <t>(-) DESPESAS BANCÁRIAS</t>
         </is>
       </c>
     </row>

</xml_diff>